<commit_message>
fix: Refactor city handling in build_results function for clarity and correctness
</commit_message>
<xml_diff>
--- a/scoring/2027/results/ASICS_2027_Scores.xlsx
+++ b/scoring/2027/results/ASICS_2027_Scores.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1308,7 +1308,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1630,7 +1630,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1906,7 +1906,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1952,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2182,7 +2182,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2366,7 +2366,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2458,7 +2458,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2734,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2872,7 +2872,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -2964,7 +2964,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3010,7 +3010,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3056,7 +3056,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3102,7 +3102,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3194,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3286,7 +3286,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3470,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3516,7 +3516,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3562,7 +3562,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3654,7 +3654,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3746,7 +3746,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3884,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4068,7 +4068,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4206,7 +4206,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4252,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4344,7 +4344,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4390,7 +4390,7 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4436,7 +4436,7 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4528,7 +4528,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4574,7 +4574,7 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4620,7 +4620,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4666,7 +4666,7 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4712,7 +4712,7 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4758,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4850,7 +4850,7 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4942,7 +4942,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5034,7 +5034,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5172,7 +5172,7 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5218,7 +5218,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5310,7 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5356,7 +5356,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>
@@ -5402,7 +5402,7 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>Bangalore</t>
+          <t>Bengaluru</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: sync main branch and preserve local AI scoring runs and results
</commit_message>
<xml_diff>
--- a/scoring/2027/results/ASICS_2027_Scores.xlsx
+++ b/scoring/2027/results/ASICS_2027_Scores.xlsx
@@ -481,17 +481,17 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1.85</v>
+        <v>1.08</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1.05</v>
+        <v>1.14</v>
       </c>
       <c r="D2">
         <f>IFERROR(ROUND(AVERAGE(B2,C2),2),"")</f>
         <v/>
       </c>
       <c r="E2" t="n">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3">
@@ -500,22 +500,18 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="B3" s="2" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>0.77</v>
       </c>
       <c r="D3">
         <f>IFERROR(ROUND(AVERAGE(B3,C3),2),"")</f>
         <v/>
       </c>
       <c r="E3" t="n">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5">
@@ -687,8 +683,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>10</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -717,10 +715,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G5" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -813,8 +809,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>3.33</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -875,8 +873,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>3.33</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -905,10 +905,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G11" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="12">
@@ -1031,10 +1029,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G15" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -1159,10 +1155,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G19" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="20">
@@ -1191,8 +1185,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G20" t="n">
-        <v>0</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1573,8 +1569,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G32" t="n">
-        <v>10</v>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1635,8 +1633,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G34" t="n">
-        <v>10</v>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1921,10 +1921,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G43" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -2145,8 +2143,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G50" t="n">
-        <v>1.67</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -2207,8 +2207,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G52" t="n">
-        <v>1.67</v>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -2269,8 +2271,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G54" t="n">
-        <v>1.67</v>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -2331,8 +2335,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G56" t="n">
-        <v>1.67</v>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -2617,10 +2623,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G65" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="66">
@@ -3061,10 +3065,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G79" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="80">
@@ -3185,10 +3187,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G83" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="84">
@@ -4611,10 +4611,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G129" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="130">
@@ -5169,10 +5167,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G147" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="148">
@@ -5553,10 +5549,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G159" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="160">
@@ -6065,10 +6059,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G175" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="176">
@@ -6253,10 +6245,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G181" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="182">
@@ -6315,10 +6305,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G183" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="184">
@@ -6377,10 +6365,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G185" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="186">
@@ -6439,10 +6425,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G187" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="188">
@@ -6821,10 +6805,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G199" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G199" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="200">
@@ -7045,8 +7027,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G206" t="n">
-        <v>5</v>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="207">
@@ -7075,10 +7059,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G207" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G207" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="208">
@@ -9709,8 +9691,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G290" t="n">
-        <v>3.75</v>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="291">
@@ -9931,8 +9915,10 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G297" t="n">
-        <v>2.5</v>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
       </c>
     </row>
     <row r="298">
@@ -10344,7 +10330,7 @@
         </is>
       </c>
       <c r="G310" t="n">
-        <v>6.25</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="311">
@@ -10788,7 +10774,7 @@
         </is>
       </c>
       <c r="G324" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
     </row>
     <row r="325">
@@ -12975,10 +12961,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G394" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G394" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="395">
@@ -13163,10 +13147,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G400" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G400" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="401">
@@ -13833,10 +13815,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G421" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G421" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="422">
@@ -14727,10 +14707,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G449" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G449" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="450">
@@ -15397,10 +15375,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G470" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G470" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="471">
@@ -15621,10 +15597,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G477" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G477" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="478">
@@ -16947,10 +16921,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G519" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G519" t="n">
+        <v>2.5</v>
       </c>
     </row>
     <row r="520">

</xml_diff>

<commit_message>
Update scored cities timestamps and modify ASICS 2027 scores file
- Changed timestamps for Bengaluru and Surat in the PARASTATAL category to "2026-10-13T17:21:32".
- Updated Surat and Bengaluru timestamps in the UPD category to "2026-10-13T17:33:44".
- Noted changes in the ASICS_2027_Scores.xlsx file, which has been modified.
</commit_message>
<xml_diff>
--- a/scoring/2027/results/ASICS_2027_Scores.xlsx
+++ b/scoring/2027/results/ASICS_2027_Scores.xlsx
@@ -481,7 +481,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1.08</v>
+        <v>2.04</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>1.14</v>
@@ -491,7 +491,7 @@
         <v/>
       </c>
       <c r="E2" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.77</v>
+        <v>1.49</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>0.77</v>
@@ -511,7 +511,7 @@
         <v/>
       </c>
       <c r="E3" t="n">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -683,10 +683,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G4" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="5">
@@ -809,10 +807,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G8" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="9">
@@ -873,10 +869,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G10" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="11">
@@ -1951,10 +1945,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G44" t="n">
+        <v>7.5</v>
       </c>
     </row>
     <row r="45">
@@ -2207,10 +2199,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G52" t="n">
+        <v>1.67</v>
       </c>
     </row>
     <row r="53">
@@ -2271,10 +2261,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G54" t="n">
+        <v>1.67</v>
       </c>
     </row>
     <row r="55">
@@ -2335,10 +2323,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G56" t="n">
+        <v>1.67</v>
       </c>
     </row>
     <row r="57">
@@ -2749,10 +2735,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G69" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="70">
@@ -4487,10 +4471,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G125" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="126">
@@ -4549,10 +4531,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G127" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="128">
@@ -4671,10 +4651,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G131" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="132">
@@ -5105,10 +5083,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G145" t="n">
+        <v>3.33</v>
       </c>
     </row>
     <row r="146">
@@ -6027,10 +6003,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G174" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="175">
@@ -6089,10 +6063,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G176" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="177">
@@ -6183,10 +6155,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G179" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="180">
@@ -6485,10 +6455,8 @@
           <t>Surat</t>
         </is>
       </c>
-      <c r="G189" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G189" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="190">
@@ -7027,10 +6995,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G206" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G206" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="207">
@@ -7153,10 +7119,8 @@
           <t>Bengaluru</t>
         </is>
       </c>
-      <c r="G210" t="inlineStr">
-        <is>
-          <t>?</t>
-        </is>
+      <c r="G210" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="211">

</xml_diff>